<commit_message>
feat: comprehensive deliverable update
PPT: 18-slide native PPTX (python-pptx, 政务蓝+金)
Tech docs: revision histories, fix architecture diagrams, Grafana HTTP fix
Project mgmt: milestone alignment, add 项目结项, cross-file consistency
Ops scripts: deploy.sh restructured (error handling), backup.sh (lock+verify), SELinux fixes, path consistency
README: reflect updated deliverables
</commit_message>
<xml_diff>
--- a/作业/交付物/项目管理/华为项目管理模板-已填写.xlsx
+++ b/作业/交付物/项目管理/华为项目管理模板-已填写.xlsx
@@ -501,6 +501,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -642,6 +643,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
@@ -744,6 +746,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -751,6 +754,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
@@ -853,6 +857,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
@@ -874,6 +879,7 @@
         </is>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
@@ -881,6 +887,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
@@ -1013,6 +1020,7 @@
         </is>
       </c>
     </row>
+    <row r="43"/>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
@@ -1081,6 +1089,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1154,6 +1163,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
@@ -2042,6 +2052,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -2070,7 +2081,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>王振光</t>
+          <t>王振光（项目经理）</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2115,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>实训实验室F4</t>
+          <t>实训实验室 F4</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2114,7 +2125,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2小时</t>
+          <t>2 小时</t>
         </is>
       </c>
     </row>
@@ -2140,6 +2151,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2150,7 +2162,10 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>明确项目方向（政务数字门户平台POC）、确定小组角色分工、讨论需求范围和技术路线、制定初步项目计划。</t>
+          <t>1. 明确项目方向和目标——政务数字门户平台 POC
+2. 确定小组角色分工（PM、Infra、App、Ops）
+3. 讨论需求范围和技术路线
+4. 制定初步项目计划</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2179,11 @@
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>企业导师（技术总监）；王振光（项目经理+架构）；胡翰斌（基础设施）；刘永涛（应用开发）；王浩乐（运维）</t>
+          <t>企业导师：技术总监，项目审批人
+王振光：项目经理+架构设计
+胡翰斌：基础设施工程师
+刘永涛：应用开发工程师
+王浩乐：运维工程师</t>
         </is>
       </c>
     </row>
@@ -2179,8 +2198,8 @@
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>1. 《实训项目概况及要求》
-2. 《业务需求规格说明书BRD简版》
-3. 《需求分析说明书SRS简版》
+2. 《业务需求规格说明书 BRD 简版》
+3. 《需求分析说明书 SRS 简版》
 4. 《华为项目管理模板》</t>
         </is>
       </c>
@@ -2195,11 +2214,19 @@
     <row r="17" ht="150" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>1. 王振光（项目经理）：介绍了项目整体框架——政务数字门户平台POC，分四个阶段（基础设施-&gt;应用部署-&gt;运维体系-&gt;文档答辩）。建议技术路线：鲲鹏ARM + FusionCompute + openEuler + Docker + Halo + MySQL + Nginx + Prometheus/Grafana。
-2. 胡翰斌（基础设施工程师）：确认FusionCompute平台可用。计划创建2台VM（2vCPU/4GB/40GB），VLAN10管理网+VLAN20业务网。预计3-4天完成基础环境搭建。
-3. 刘永涛（应用开发工程师）：建议使用Halo v2.x（国产开源、支持Markdown），WordPress备选。Docker Compose编排Halo+MySQL+Nginx三个服务。需确认ARM64镜像兼容性。
-4. 王浩乐（运维工程师）：运维四件事——Nginx HTTPS代理、Prometheus+Grafana监控、backup.sh自动备份、deploy.sh一键部署。监控大盘至少含CPU/内存/磁盘/容器状态。
-5. 企业导师：强调文档记录重要性（至少4次纪要）、大节点做VM快照、优先考虑国产化兼容性、中期汇报定在第3周。</t>
+          <t>1. 王振光（项目经理）：
+介绍了项目的整体框架：政务数字门户平台是一个面向政企客户的技术博客系统 POC，需要在鲲鹏 ARM 架构上使用容器化部署。项目分为四个阶段——基础设施搭建、应用开发部署、运维体系构建、文档与答辩。建议技术路线为：FusionCompute + openEuler + Docker + Halo + MySQL + Nginx + Prometheus/Grafana。
+2. 胡翰斌（基础设施工程师）：
+确认 FusionCompute 平台可用性。计划先在 FC 上创建集群（BlogOps-Cluster），部署 2 台 VM（2vCPU/4GB/40GB，openEuler 22.03 LTS ARM）。网络规划：VLAN 10 用于管理（192.168.10.0/24），VLAN 20 用于业务（192.168.20.0/24）。预计 3-4 天完成基础环境搭建。
+3. 刘永涛（应用开发工程师）：
+建议使用 Halo v2.x 作为博客系统（国产开源、支持 Markdown、云原生友好），WordPress 作为备选。应用以容器方式运行，编写 Docker Compose 编排 Halo + MySQL + Nginx 三个服务。需要确认 ARM64 架构下的镜像兼容性。
+4. 王浩乐（运维工程师）：
+提出运维要做四件事：Nginx HTTPS 反向代理、Prometheus+Grafana 监控、数据库每日自动备份（backup.sh + crontab）、一键部署脚本（deploy.sh）。建议监控大盘至少包含 CPU/内存/磁盘/容器状态。
+5. 企业导师：
+强调文档的重要性——每个阶段都要有记录，会议纪要至少 4 次
+提醒大家每次大节点做 VM 快照，方便回滚
+建议技术选型优先考虑国产化兼容性
+中期汇报定在第3周，最终答辩在第4周末</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2240,11 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>1. 项目名称确认：政务数字门户平台POC（DMP-2026-001）
-2. 技术栈确认：鲲鹏ARM + FusionCompute + openEuler + Docker + Halo + MySQL + Nginx + Prometheus/Grafana
+          <t>1. 项目名称确认：政务数字门户平台 POC（DMP-2026-001）
+2. 技术栈确认：鲲鹏 ARM + FusionCompute + openEuler + Docker + Halo + MySQL + Nginx + Prometheus/Grafana
 3. 角色分工确认：王振光（PM+架构）、胡翰斌（Infra）、刘永涛（App）、王浩乐（Ops）
 4. 第一周目标：完成基础设施搭建（VM创建 + Docker安装 + 网络配置）
-5. 下次会议：2026年6月14日小组周会</t>
+5. 下次会议时间：2026年6月14日（周日）小组周会</t>
         </is>
       </c>
     </row>
@@ -2290,6 +2317,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -2318,7 +2346,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>王振光</t>
+          <t>王振光（项目经理）</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2380,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>实训实验室F4</t>
+          <t>实训实验室 F4</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2362,7 +2390,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1小时30分钟</t>
+          <t>1 小时 30 分钟</t>
         </is>
       </c>
     </row>
@@ -2388,6 +2416,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2398,7 +2427,10 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>检查第一周基础设施搭建进度、确认Docker和网络配置完成情况、规划第二周应用部署工作、识别阻塞问题。</t>
+          <t>1. 检查第一周基础设施搭建进度
+2. 确认 Docker 环境安装和网络配置完成情况
+3. 规划第二周应用部署工作
+4. 识别和解决阻塞问题</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2444,11 @@
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>企业导师（技术总监）；王振光（PM）；胡翰斌（Infra）；刘永涛（App）；王浩乐（Ops）</t>
+          <t>企业导师：技术总监
+王振光：项目经理+架构设计
+胡翰斌：基础设施工程师
+刘永涛：应用开发工程师
+王浩乐：运维工程师</t>
         </is>
       </c>
     </row>
@@ -2427,8 +2463,8 @@
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>1. 第1周工作进度汇报
-2. VM配置清单和网络拓扑草图
-3. Docker安装验证截图</t>
+2. VM 配置清单和网络拓扑草图
+3. Docker 安装验证截图</t>
         </is>
       </c>
     </row>
@@ -2442,17 +2478,35 @@
     <row r="17" ht="240" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>1. 胡翰斌（基础设施工程师）：汇报第1周完成情况：
-✅ FC集群BlogOps-Cluster创建完成，鲲鹏TaiShan 200
-✅ 2台VM创建（2vCPU/4GB/40GB），openEuler 22.03 LTS SP2安装完毕，uname -m确认aarch64
-✅ VLAN 10（管理网）和VLAN 20（业务网）划分完成
-✅ 安全组仅开放22/80/443端口
-✅ Docker CE 24.x安装完成，systemd自启动配置完毕
-⚠️ 遇到问题：Docker Hub镜像拉取速度慢（国内网络），建议配置镜像加速或准备离线镜像
-2. 刘永涛（应用开发工程师）：已完成Halo v2.x技术调研，确认支持ARM64。docker-compose.yml初版已编写，Nginx反向代理配置模板已准备。问题：需解决Docker Hub网络问题。
-3. 王浩乐（运维工程师）：已调研Prometheus + Grafana技术方案，Nginx SSL配置方案准备就绪。需等待应用部署后才能开始监控配置。
-4. 王振光（项目经理）：总体进度正常。针对Docker Hub慢，建议阿里云镜像加速+离线镜像两种方案并行。系统架构设计初稿已出。提醒做VM快照。
-5. 企业导师：第一周完成得很好。建议在docker-compose.yml中标注配置含义。中期汇报要在第3周展示可访问的博客系统+基本运维能力。</t>
+          <t>1. 胡翰斌（基础设施工程师）：
+汇报第1周完成情况：
+✅ FusionCompute 集群 BlogOps-Cluster 创建完成，主机为鲲鹏 TaiShan 200
+✅ 2 台 VM 创建完成（2vCPU/4GB/40GB），openEuler 22.03 LTS SP2 安装完毕，uname -m 确认显示 aarch64
+✅ VLAN 10（管理网 192.168.10.0/24）和 VLAN 20（业务网 192.168.20.0/24）划分完成
+✅ 安全组仅开放 22/80/443 端口，从管理网无法直接 telnet DB 3306 端口
+✅ Docker CE 24.x 安装完成，systemd 自启动配置完毕
+⚠️ 遇到问题：Docker Hub 镜像拉取速度较慢（国内网络），建议配置镜像加速器或准备离线镜像
+📋 下周计划：协助刘永涛完成 Harbor/Harbor-alternative 镜像仓库搭建
+2. 刘永涛（应用开发工程师）：
+已完成 Halo v2.x 的技术调研，确认支持 ARM64 架构
+已完成 docker-compose.yml 初版编写，待测试
+已准备好 Nginx 反向代理配置模板
+⚠️ 问题：Halo 官方镜像需要从 Docker Hub 拉取，需要胡翰斌配合解决网络问题
+📋 下周计划：完成 Docker Compose 编排，实现 Halo + MySQL + Nginx 部署上线
+3. 王浩乐（运维工程师）：
+已调研 Prometheus + Grafana + node_exporter + cAdvisor 技术方案
+已完成 Nginx SSL 配置方案（自签名证书用于 POC）
+⚠️ 需要等到应用部署后才能开始监控配置
+📋 下周计划：应用上线后立即配置 Nginx HTTPS、开始搭建监控
+4. 王振光（项目经理）：
+整体进度正常，符合计划
+针对 Docker Hub 慢的问题，建议两种方案并行：(1) 配置阿里云容器镜像加速器；(2) 准备离线镜像包
+已完成的系统架构设计初稿请大家审阅
+提醒大家做 VM 快照（基础设施就绪这个节点很重要）
+5. 企业导师：
+第一周基础设施完成的很好
+建议在 docker-compose.yml 中明确标注每个配置项的含义，方便后续写文档
+提醒：中期汇报要在第3周进行，需展示一个可访问的博客系统 + 基本运维能力</t>
         </is>
       </c>
     </row>
@@ -2466,10 +2520,10 @@
     <row r="19" ht="80" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>1. Docker Hub加速方案：配置阿里云镜像加速器（daemon.json），同时准备离线镜像
-2. 第二周目标：完成应用部署上线（Halo博客可通过浏览器访问）
-3. VM快照：会后立即做 Week1-Infra-Ready 快照
-4. 下次会议：2026年6月21日</t>
+          <t>1. Docker Hub 加速方案：配置阿里云镜像加速器（daemon.json），同时准备离线镜像
+2. 第二周目标：完成应用部署上线（Halo 博客可通过浏览器访问）
+3. VM 快照：会后立即对当前状态做快照，命名 `Week1-Infra-Ready`
+4. 下次会议：2026年6月21日（周日）——重点检查应用部署和运维配置进展</t>
         </is>
       </c>
     </row>
@@ -2541,6 +2595,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -2559,7 +2614,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>第2周周会——应用部署完成及运维体系启动</t>
+          <t>第2周周会——应用部署完成 &amp; 运维体系启动</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2569,7 +2624,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>王振光</t>
+          <t>王振光（项目经理）</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2658,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>实训实验室F4</t>
+          <t>实训实验室 F4</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2613,7 +2668,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2小时</t>
+          <t>2 小时</t>
         </is>
       </c>
     </row>
@@ -2639,6 +2694,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2649,7 +2705,10 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>演示应用部署成果（博客系统线上可访问）、启动运维体系建设、准备中期汇报内容、识别遗留问题。</t>
+          <t>1. 演示应用部署成果（博客系统线上可访问）
+2. 启动运维体系建设（监控、备份、一键部署）
+3. 准备中期汇报内容
+4. 识别遗留问题和风险</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2722,11 @@
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>企业导师（技术总监）；王振光（PM）；胡翰斌（Infra）；刘永涛（App）；王浩乐（Ops）</t>
+          <t>企业导师：技术总监
+王振光：项目经理+架构设计
+胡翰斌：基础设施工程师
+刘永涛：应用开发工程师
+王浩乐：运维工程师</t>
         </is>
       </c>
     </row>
@@ -2677,9 +2740,9 @@
     <row r="15" ht="80" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>1. 应用部署完成截图（Halo首页+后台+Docker ps）
-2. Docker Compose编排文件
-3. Nginx配置（含SSL跳转）
+          <t>1. 应用部署完成截图（Halo 首页 + 后台 + Docker ps）
+2. Docker Compose 编排文件
+3. Nginx 配置（含 SSL 跳转）
 4. 中期汇报PPT初稿</t>
         </is>
       </c>
@@ -2694,24 +2757,37 @@
     <row r="17" ht="345" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>1. 刘永涛（应用开发工程师）：汇报第2周完成情况：
-✅ docker-compose.yml编排完成，halo+mysql+nginx三个服务
-✅ Halo v2.x部署成功，浏览器访问正常
-✅ MySQL数据持久化验证通过（docker rm -f mysql后数据不丢）
-✅ Nginx反向代理+80-&gt;443强制跳转
-✅ 博客功能完整：Markdown/代码高亮/分类/标签/搜索/评论
-✅ 审核工作流配置完成：草稿-&gt;审核-&gt;通过/驳回
-⚠️ 自签名证书浏览器显示不安全警告（POC阶段可接受）
+          <t>1. 刘永涛（应用开发工程师）：
+汇报第2周完成情况：
+✅ docker-compose.yml 编排完成，包含 halo、mysql、nginx 三个服务
+✅ Halo v2.x 博客成功部署，浏览器访问 http://192.168.20.x 正常显示首页
+✅ MySQL 8.0 数据持久化至宿主机 /data/mysql，验证过 docker rm -f mysql 后数据不丢失
+✅ Nginx 反向代理配置完成，80→443 强制跳转
+✅ 博客功能验证：Markdown发布、代码高亮、分类标签、全文搜索、评论均正常
+✅ 审核工作流配置完成：默认草稿→审核员可执行通过/驳回→通过后前台可见
+⚠️ 当前使用自签名证书，浏览器显示"不安全"警告（POC 阶段可接受）
+📋 协助王浩乐完成运维配置
 2. 王浩乐（运维工程师）：
-✅ Prometheus + cAdvisor部署完成，Targets全部UP
-✅ Grafana监控大盘导入，展示CPU/内存/磁盘/容器状态
-✅ backup.sh编写完毕：每日02:00 mysqldump，保留7天
-🔄 deploy.sh开发中——已完成框架，当前耗时35分钟需优化（目标≤30分钟）
+✅ Prometheus + node_exporter + cAdvisor 部署完成，Targets 全部 UP
+✅ Grafana 容器监控大盘导入，展示 CPU/内存/磁盘/网络/容器状态
+✅ backup.sh 编写完毕：mysqldump 每日 02:00 执行，保留 7 天，存储至 /data/backup/
+🔄 deploy.sh 一键部署脚本开发中——已完成框架，正在测试全流程耗时
+⚠️ 当前一键部署耗时约 35 分钟，需优化镜像拉取环节（目标 ≤30 分钟）
+📋 下周计划：优化 deploy.sh 效率、完成性能压测
 3. 胡翰斌（基础设施工程师）：
-✅ 阿里云镜像加速器配置完成，镜像拉取从30分钟降至5分钟
-✅ 私有Registry备用仓库搭建完成
-4. 王振光（项目经理）：整体进度略微超前。中期汇报内容框架：项目概述-&gt;架构展示-&gt;Live Demo-&gt;当前进展-&gt;下一步计划。本周五中期汇报演练。
-5. 企业导师：应用部署效果不错。建议中期汇报重点展示容器化部署灵活性、数据持久化验证、监控大盘。文档格式要符合模板要求。</t>
+✅ 协助解决 Docker Hub 慢的问题：配置阿里云镜像加速器，镜像拉取速度从 30 分钟降至 5 分钟
+✅ 私有镜像仓库（Registry）搭好备用
+🔄 在协助王浩乐优化 deploy.sh，考虑预置镜像减少拉取时间
+📋 下周计划：虚拟机快照、协助压测
+4. 王振光（项目经理）：
+整体进度略微超前，应用上线比计划提前了几天
+中期汇报内容框架已拟定：项目概述→架构展示→Live Demo→当前进展→下一步计划
+提醒：第4周需要留足文档和答辩准备时间
+本周五（6/26）进行中期汇报演练
+5. 企业导师：
+应用部署效果不错，博客功能完整
+建议中期汇报时重点展示：①容器化部署的灵活性（docker compose up -d 一键启动）；②数据持久化验证（删容器不丢数据）；③监控大盘
+提醒：文档格式要符合模板要求，截图要清晰</t>
         </is>
       </c>
     </row>
@@ -2725,11 +2801,11 @@
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>1. deploy.sh优化目标：压缩至30分钟内（预拉取镜像）
-2. VM快照：会后做 Week2-App-Live 快照
-3. 中期汇报排练：6月26日上午完整演练
-4. 下周重点：运维体系完善+性能压测+文档撰写
-5. 下次会议：2026年6月28日</t>
+          <t>1. deploy.sh 优化目标：将一键部署耗时压缩至 30 分钟内（通过预拉取镜像或使用本地仓库）
+2. VM 快照：会后立即做 `Week2-App-Live` 快照
+3. 中期汇报排练：6月26日（周五）上午进行完整演练
+4. 下周重点：运维体系完善 + 性能压测 + 文档撰写
+5. 下次会议：2026年6月28日（周日）——中期汇报总结 &amp; 文档交付准备</t>
         </is>
       </c>
     </row>
@@ -2801,6 +2877,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -2819,7 +2896,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>第3周周会——中期汇报复盘及文档交付准备</t>
+          <t>第3周周会——中期汇报复盘 &amp; 文档交付准备</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2829,7 +2906,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>王振光</t>
+          <t>王振光（项目经理）</t>
         </is>
       </c>
     </row>
@@ -2863,7 +2940,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>实训实验室F4</t>
+          <t>实训实验室 F4</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -2873,7 +2950,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2小时</t>
+          <t>2 小时</t>
         </is>
       </c>
     </row>
@@ -2899,6 +2976,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -2909,7 +2987,11 @@
     <row r="11" ht="80" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>复盘中期汇报、确认运维体系全部就绪、性能和安全测试结果评审、分配文档写作任务、制定最终答辩策略。</t>
+          <t>1. 复盘中期汇报，整理导师反馈
+2. 确认运维体系全部就绪
+3. 性能压测和安全测试结果评审
+4. 分配文档写作任务，确保第4周完成
+5. 制定最终答辩策略</t>
         </is>
       </c>
     </row>
@@ -2923,7 +3005,11 @@
     <row r="13" ht="80" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>企业导师（技术总监）；王振光（PM）；胡翰斌（Infra）；刘永涛（App）；王浩乐（Ops）</t>
+          <t>企业导师：技术总监
+王振光：项目经理+架构设计
+胡翰斌：基础设施工程师
+刘永涛：应用开发工程师
+王浩乐：运维工程师</t>
         </is>
       </c>
     </row>
@@ -2938,8 +3024,8 @@
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>1. 中期汇报PPT和演示录像
-2. 性能压测报告（ab+JMeter）
-3. 运维脚本终版（deploy.sh+backup.sh）
+2. 性能压测报告（ab + JMeter）
+3. 运维脚本终版（deploy.sh + backup.sh）
 4. 技术文档初稿</t>
         </is>
       </c>
@@ -2954,27 +3040,43 @@
     <row r="17" ht="390" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>1. 王振光（项目经理）：复盘6月26日中期汇报情况：
-✅ 博客系统Live Demo流畅，访问正常
-✅ 容器化演示——docker compose up -d一键启动
-✅ 监控大盘展示完整——实时CPU/内存/容器状态
-✅ 数据持久化验证——删容器不丢数据
-⚠️ 导师反馈：HTTPS自签名证书有警告，建议标注POC阶段说明
-⚠️ 导师反馈：答辩应更强调"国产化"和"可复制性"两个亮点
+          <t>1. 王振光（项目经理）：
+复盘了 6月26日的中期汇报情况：
+✅ 博客系统 Live Demo 流畅，访问正常
+✅ 容器化部署演示顺利——docker compose up -d 一键启动 3 个服务
+✅ 监控大盘展示完整——实时 CPU/内存/容器状态可视化
+✅ 数据持久化验证——docker rm -f mysql 后数据恢复正常
+⚠️ 导师反馈：HTTPS 用的是自签名证书，浏览器有警告，建议标注"POC阶段说明"
+⚠️ 导师反馈：答辩时应更强调"国产化"和"可复制性"两个亮点
+📋 最终答辩要突出技术深度和实际价值，不只展示功能
 2. 王浩乐（运维工程师）：
-✅ deploy.sh优化完成！全流程28分钟（≤30分钟目标达成）
-✅ backup.sh验证通过：模拟故障-&gt;恢复-&gt;数据完整
-✅ 性能压测达标：95分位响应2.1秒（目标≤3秒），50并发错误率0%
-✅ JMeter验证TPS约28（目标≥20）
-✅ 安全测试通过：管理网无法访问3306，安全组拦截生效
+✅ deploy.sh 一键部署脚本优化完成！全流程耗时 28 分钟（≤30分钟目标达成）
+优化措施：Docker 镜像预拉取 + 阿里云加速器
+测试环境：全新 openEuler 22.03 VM，从零到博客可访问
+✅ backup.sh 验证通过：模拟 MySQL 故障→从备份恢复→数据完整
+✅ Prometheus + Grafana 监控运行稳定，容器重启后自动恢复
+✅ 性能压测结果：ab -n 1000 -c 50 → 95分位响应 2.1秒（目标 ≤3秒，达标）
+✅ JMeter 50并发测试：错误率 0%，TPS 约 28（目标 ≥20，达标）
+✅ 安全测试：管理网无法访问 3306，未授权访问被安全组拦截
 3. 刘永涛（应用开发工程师）：
-✅ 全部功能测试通过（发布/审核/搜索/评论/代码高亮）
-✅ 兼容性测试：Chrome/Firefox/Edge均正常
-🔄 部署实施手册已完成70%
+✅ 博客全部功能测试通过（发布/审核/搜索/评论/代码高亮/全文检索）
+✅ 兼容性测试：Chrome 120+、Firefox 121+、Edge 120+ 正常
+✅ 响应式布局正常（桌面+平板+手机）
+🔄 协助编写部署实施手册（已完成70%）
+📋 本周完成部署实施手册定稿
 4. 胡翰斌（基础设施工程师）：
-✅ VM快照：Week1/Week2/Week3三个节点已保存
-✅ 验证快照回滚正常，磁盘使用率45%
-5. 企业导师：中期汇报技术实现扎实。最终答辩突出三个亮点——国产化全栈、容器化可复制性、运维完备性。答辩15分钟演示+5分钟问答。</t>
+✅ 已做 VM 快照：`Week1-Infra-Ready`、`Week2-App-Live`、`Week3-Ops-Ready` 三个节点
+✅ 验证快照回滚正常
+✅ 磁盘使用率 45%（100GB 数据盘，剩余充足）
+📋 最终答辩前再做一次完整快照
+5. 企业导师：
+中期汇报整体不错，技术实现扎实
+最终答辩建议突出 3 个亮点：
+1. **国产化全栈**：鲲鹏 ARM + FusionCompute + openEuler——完全自主可控
+2. **容器化可复制**：deploy.sh 30分钟内一键部署到新环境——体现交付能力
+3. **运维完备性**：监控+备份+恢复——不只是"能跑"，而是"可维护"
+文档不要堆砌截图，要有逻辑：为什么这样设计→怎么做→结果如何
+答辩时间控制在 15 分钟演示 + 5 分钟问答</t>
         </is>
       </c>
     </row>
@@ -2990,13 +3092,13 @@
         <is>
           <t>1. 最终答辩重点：国产化全栈 + 容器化可复制性 + 运维完备性
 2. 文档分工：
-   - 王振光：架构设计说明书、答辩PPT
-   - 胡翰斌：协助架构章节、VM配置部分
-   - 刘永涛：部署实施手册
-   - 王浩乐：运维操作手册
-3. 文档交付截止：7月2日定稿
+王振光：架构设计说明书、答辩PPT
+胡翰斌：协助架构章节、VM配置部分
+刘永涛：部署实施手册
+王浩乐：运维操作手册
+3. 文档交付截止：7月2日前定稿
 4. 答辩排练：7月2日下午完整演练
-5. VM快照：最终快照 Final-PreDefense</t>
+5. VM快照：文档定稿后做最终快照 `Final-PreDefense`</t>
         </is>
       </c>
     </row>

</xml_diff>